<commit_message>
Obtener proyeccion metas y contribuciones hasta agosto de 2026
</commit_message>
<xml_diff>
--- a/main_data/contrafactual_num_vinculaciones.xlsx
+++ b/main_data/contrafactual_num_vinculaciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Predecido</t>
+          <t>Contrafactual</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -466,180 +466,854 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45658</v>
+        <v>44562</v>
       </c>
       <c r="B2" t="n">
-        <v>313104.1999999998</v>
+        <v>2830.230538779878</v>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>313674</v>
+        <v>2756</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45689</v>
+        <v>44593</v>
       </c>
       <c r="B3" t="n">
-        <v>318181.2999999998</v>
+        <v>6507.788293912484</v>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>317970</v>
+        <v>6346</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45717</v>
+        <v>44621</v>
       </c>
       <c r="B4" t="n">
-        <v>323258.3999999998</v>
+        <v>10844.84735149614</v>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>322701</v>
+        <v>11127</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45748</v>
+        <v>44652</v>
       </c>
       <c r="B5" t="n">
-        <v>328335.4999999999</v>
+        <v>14521.21828366955</v>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>327805</v>
+        <v>15050</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45778</v>
+        <v>44682</v>
       </c>
       <c r="B6" t="n">
-        <v>333412.5999999999</v>
+        <v>18913.94976773481</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>334142</v>
+        <v>19497</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45809</v>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="n">
-        <v>338489.7</v>
-      </c>
+        <v>44713</v>
+      </c>
+      <c r="B7" t="n">
+        <v>23166.26322801862</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>340333</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1843.300000000047</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.005445660532654455</v>
-      </c>
+        <v>23697</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45839</v>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="n">
-        <v>343566.8</v>
-      </c>
+        <v>44743</v>
+      </c>
+      <c r="B8" t="n">
+        <v>27870.35121940427</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>348209</v>
-      </c>
-      <c r="E8" t="n">
-        <v>4642.200000000012</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.01351178286144066</v>
-      </c>
+        <v>27788</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45870</v>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="n">
-        <v>348643.9</v>
-      </c>
+        <v>44774</v>
+      </c>
+      <c r="B9" t="n">
+        <v>32776.56452580648</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>358830</v>
-      </c>
-      <c r="E9" t="n">
-        <v>10186.09999999998</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.02921634366756446</v>
-      </c>
+        <v>32611</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45901</v>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="n">
-        <v>353721.0000000001</v>
-      </c>
+        <v>44805</v>
+      </c>
+      <c r="B10" t="n">
+        <v>38226.17188921632</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>377185</v>
-      </c>
-      <c r="E10" t="n">
-        <v>23463.99999999994</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.06633476666638378</v>
-      </c>
+        <v>37558</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45931</v>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="n">
-        <v>358798.1000000001</v>
-      </c>
+        <v>44835</v>
+      </c>
+      <c r="B11" t="n">
+        <v>43654.94282680413</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>393365</v>
-      </c>
-      <c r="E11" t="n">
-        <v>34566.89999999991</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.09634081116928964</v>
-      </c>
+        <v>42447</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
+        <v>44866</v>
+      </c>
+      <c r="B12" t="n">
+        <v>49443.71254583978</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>47450</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>44896</v>
+      </c>
+      <c r="B13" t="n">
+        <v>54613.53935038361</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>51480</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>44927</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3410.138666556948</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>3491</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>44958</v>
+      </c>
+      <c r="B15" t="n">
+        <v>7671.149656315024</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>7365</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>44986</v>
+      </c>
+      <c r="B16" t="n">
+        <v>12506.25545166416</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>12175</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>45017</v>
+      </c>
+      <c r="B17" t="n">
+        <v>16382.63360711225</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>16181</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>45047</v>
+      </c>
+      <c r="B18" t="n">
+        <v>20875.63567013169</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>21293</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>45078</v>
+      </c>
+      <c r="B19" t="n">
+        <v>25014.41075539099</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>25969</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>45108</v>
+      </c>
+      <c r="B20" t="n">
+        <v>29441.06694256765</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>30959</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>45139</v>
+      </c>
+      <c r="B21" t="n">
+        <v>33872.81942614278</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="n">
+        <v>35412</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>45170</v>
+      </c>
+      <c r="B22" t="n">
+        <v>38647.86762914677</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="n">
+        <v>39977</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>45200</v>
+      </c>
+      <c r="B23" t="n">
+        <v>43179.23713797318</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>44622</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>45231</v>
+      </c>
+      <c r="B24" t="n">
+        <v>47844.21431779443</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>49728</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>45261</v>
+      </c>
+      <c r="B25" t="n">
+        <v>51700.58889045163</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>53417</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>45292</v>
+      </c>
+      <c r="B26" t="n">
+        <v>3158.231922376057</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>3144</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>45323</v>
+      </c>
+      <c r="B27" t="n">
+        <v>6950.39117998117</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>7236</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>45352</v>
+      </c>
+      <c r="B28" t="n">
+        <v>11085.4391081266</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>10666</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B29" t="n">
+        <v>14206.46863166847</v>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>13864</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>45413</v>
+      </c>
+      <c r="B30" t="n">
+        <v>17710.01543951868</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>16810</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>45444</v>
+      </c>
+      <c r="B31" t="n">
+        <v>20760.90689705006</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>19493</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>45474</v>
+      </c>
+      <c r="B32" t="n">
+        <v>23904.87083324858</v>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>22743</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>45505</v>
+      </c>
+      <c r="B33" t="n">
+        <v>26906.73592293336</v>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>25820</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>45536</v>
+      </c>
+      <c r="B34" t="n">
+        <v>30033.91997246678</v>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>29526</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>45566</v>
+      </c>
+      <c r="B35" t="n">
+        <v>32827.5340337749</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>32639</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>45597</v>
+      </c>
+      <c r="B36" t="n">
+        <v>35585.21015258514</v>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>35619</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>45627</v>
+      </c>
+      <c r="B37" t="n">
+        <v>37619.44728761322</v>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>38529</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>45658</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2248.214540590253</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="n">
+        <v>2264</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>45689</v>
+      </c>
+      <c r="B39" t="n">
+        <v>4840.383750590993</v>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>4955</v>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>45717</v>
+      </c>
+      <c r="B40" t="n">
+        <v>7552.665657965811</v>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="n">
+        <v>7842</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>45748</v>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="n">
+        <v>9469.135005711065</v>
+      </c>
+      <c r="D41" t="n">
+        <v>11159</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1689.864994288935</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.1514351639294682</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>45778</v>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="n">
+        <v>11548.34964554838</v>
+      </c>
+      <c r="D42" t="n">
+        <v>14390</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2841.65035445162</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.1974739648680764</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>45809</v>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="n">
+        <v>13244.1508358534</v>
+      </c>
+      <c r="D43" t="n">
+        <v>17541</v>
+      </c>
+      <c r="E43" t="n">
+        <v>4296.849164146601</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.2449603308902914</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>45839</v>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="n">
+        <v>14919.04457619315</v>
+      </c>
+      <c r="D44" t="n">
+        <v>21240</v>
+      </c>
+      <c r="E44" t="n">
+        <v>6320.955423806847</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.2975967713656708</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>45870</v>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="n">
+        <v>16428.29297760444</v>
+      </c>
+      <c r="D45" t="n">
+        <v>24210</v>
+      </c>
+      <c r="E45" t="n">
+        <v>7781.707022395556</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.3214253210407086</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="n">
+        <v>17939.90979472605</v>
+      </c>
+      <c r="D46" t="n">
+        <v>27850</v>
+      </c>
+      <c r="E46" t="n">
+        <v>9910.090205273948</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.3558380684119909</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="n">
+        <v>19183.29956814164</v>
+      </c>
+      <c r="D47" t="n">
+        <v>31609</v>
+      </c>
+      <c r="E47" t="n">
+        <v>12425.70043185836</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.3931064074111284</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
         <v>45962</v>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="n">
-        <v>363875.2000000001</v>
-      </c>
-      <c r="D12" t="n">
-        <v>408348</v>
-      </c>
-      <c r="E12" t="n">
-        <v>44472.79999999987</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.1222199259526339</v>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="n">
+        <v>20343.76808464343</v>
+      </c>
+      <c r="D48" t="n">
+        <v>34893</v>
+      </c>
+      <c r="E48" t="n">
+        <v>14549.23191535657</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.4169670683333784</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="n">
+        <v>21040.25915120763</v>
+      </c>
+      <c r="D49" t="n">
+        <v>38305</v>
+      </c>
+      <c r="E49" t="n">
+        <v>17264.74084879237</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.4507176830385687</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="n">
+        <v>1230.136314295369</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2669</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1438.863685704631</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.5391021677424621</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="n">
+        <v>2591.027927542779</v>
+      </c>
+      <c r="D51" t="n">
+        <v>5869</v>
+      </c>
+      <c r="E51" t="n">
+        <v>3277.972072457221</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.5585230997541695</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="n">
+        <v>3955.208407937015</v>
+      </c>
+      <c r="D52" t="n">
+        <v>9756</v>
+      </c>
+      <c r="E52" t="n">
+        <v>5800.791592062985</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.5945870840572965</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="n">
+        <v>4851.278798864098</v>
+      </c>
+      <c r="D53" t="n">
+        <v>13495</v>
+      </c>
+      <c r="E53" t="n">
+        <v>8643.721201135902</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.6405128715180365</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="n">
+        <v>5788.18845326321</v>
+      </c>
+      <c r="D54" t="n">
+        <v>16859</v>
+      </c>
+      <c r="E54" t="n">
+        <v>11070.81154673679</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.6566707127787407</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="n">
+        <v>6494.170240231875</v>
+      </c>
+      <c r="D55" t="n">
+        <v>19966</v>
+      </c>
+      <c r="E55" t="n">
+        <v>13471.82975976812</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.6747385435123773</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="n">
+        <v>7156.775190368924</v>
+      </c>
+      <c r="D56" t="n">
+        <v>23778</v>
+      </c>
+      <c r="E56" t="n">
+        <v>16621.22480963108</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.6990169404336394</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="n">
+        <v>7709.844447218628</v>
+      </c>
+      <c r="D57" t="n">
+        <v>27426</v>
+      </c>
+      <c r="E57" t="n">
+        <v>19716.15555278137</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.718885566717034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>